<commit_message>
Update phase 0.5 review workbook
</commit_message>
<xml_diff>
--- a/docs/phase-0.5-review.xlsx
+++ b/docs/phase-0.5-review.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/henryyeh/dev/fitness-mcp/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86CEEA9C-5564-E449-AF53-9B05C75589B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B82E2F1A-41A9-004A-8D3F-52BCC17BD6D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="25600" windowHeight="15400" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="25600" windowHeight="15400" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="使用說明" sheetId="1" r:id="rId1"/>

</xml_diff>